<commit_message>
Add ranked items with historical basket transition
Import 20 validated trade candidates, weight them from their first complete
HaloSkins scan, and preserve longer-range chart continuity with the actual
pre-transition contribution applied to all marketplace lines.

Co-Authored-By: Claude Haiku 4.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/basket.xlsx
+++ b/data/basket.xlsx
@@ -560,7 +560,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
@@ -594,16 +594,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -637,6 +633,10 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="49"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
@@ -1104,7 +1104,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA41"/>
+  <dimension ref="A1:AA61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="8" customWidth="1" style="28" min="1" max="1"/>
@@ -6190,6 +6190,2506 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="43" t="inlineStr">
+        <is>
+          <t>Sealed Dead Hand Terminal</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>21055.061911904</v>
+      </c>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/sealed-dead-hand-terminal/normal</t>
+        </is>
+      </c>
+      <c r="F42" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/container/sealed-dead-hand-terminal</t>
+        </is>
+      </c>
+      <c r="G42" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/sealed-dead-hand-terminal</t>
+        </is>
+      </c>
+      <c r="H42" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=Sealed+Dead+Hand+Terminal</t>
+        </is>
+      </c>
+      <c r="I42" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/Sealed%20Dead%20Hand%20Terminal</t>
+        </is>
+      </c>
+      <c r="J42" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/sealed-dead-hand-terminal</t>
+        </is>
+      </c>
+      <c r="K42" s="44" t="n"/>
+      <c r="L42" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=Sealed+Dead+Hand+Terminal&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=normal</t>
+        </is>
+      </c>
+      <c r="M42" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=Sealed+Dead+Hand+Terminal</t>
+        </is>
+      </c>
+      <c r="N42" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/sealed-dead-hand-terminal?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=normal</t>
+        </is>
+      </c>
+      <c r="O42" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/sealed-dead-hand-terminal</t>
+        </is>
+      </c>
+      <c r="P42" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/sealed-dead-hand-terminal/</t>
+        </is>
+      </c>
+      <c r="Q42" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/Sealed%20Dead%20Hand%20Terminal</t>
+        </is>
+      </c>
+      <c r="R42" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=Sealed+Dead+Hand+Terminal&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S42" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/sealed-dead-hand-terminal/</t>
+        </is>
+      </c>
+      <c r="T42" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=Sealed+Dead+Hand+Terminal</t>
+        </is>
+      </c>
+      <c r="U42" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=Sealed+Dead+Hand+Terminal</t>
+        </is>
+      </c>
+      <c r="V42" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/sealed-dead-hand-terminal</t>
+        </is>
+      </c>
+      <c r="W42" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/sealed-dead-hand-terminal</t>
+        </is>
+      </c>
+      <c r="X42" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/Sealed%20Dead%20Hand%20Terminal</t>
+        </is>
+      </c>
+      <c r="Y42" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=Sealed+Dead+Hand+Terminal</t>
+        </is>
+      </c>
+      <c r="Z42" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/Sealed-Dead-Hand-Terminal</t>
+        </is>
+      </c>
+      <c r="AA42" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=Sealed+Dead+Hand+Terminal&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="43" t="inlineStr">
+        <is>
+          <t>Sealed Genesis Terminal</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>2162.683902624</v>
+      </c>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/sealed-genesis-terminal/normal</t>
+        </is>
+      </c>
+      <c r="F43" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/container/sealed-genesis-terminal</t>
+        </is>
+      </c>
+      <c r="G43" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/sealed-genesis-terminal</t>
+        </is>
+      </c>
+      <c r="H43" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=Sealed+Genesis+Terminal</t>
+        </is>
+      </c>
+      <c r="I43" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/Sealed%20Genesis%20Terminal</t>
+        </is>
+      </c>
+      <c r="J43" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/sealed-genesis-terminal</t>
+        </is>
+      </c>
+      <c r="K43" s="44" t="n"/>
+      <c r="L43" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=Sealed+Genesis+Terminal&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=normal</t>
+        </is>
+      </c>
+      <c r="M43" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=Sealed+Genesis+Terminal</t>
+        </is>
+      </c>
+      <c r="N43" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/sealed-genesis-terminal?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=normal</t>
+        </is>
+      </c>
+      <c r="O43" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/sealed-genesis-terminal</t>
+        </is>
+      </c>
+      <c r="P43" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/sealed-genesis-terminal/</t>
+        </is>
+      </c>
+      <c r="Q43" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/Sealed%20Genesis%20Terminal</t>
+        </is>
+      </c>
+      <c r="R43" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=Sealed+Genesis+Terminal&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S43" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/sealed-genesis-terminal/</t>
+        </is>
+      </c>
+      <c r="T43" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=Sealed+Genesis+Terminal</t>
+        </is>
+      </c>
+      <c r="U43" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=Sealed+Genesis+Terminal</t>
+        </is>
+      </c>
+      <c r="V43" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/sealed-genesis-terminal</t>
+        </is>
+      </c>
+      <c r="W43" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/sealed-genesis-terminal</t>
+        </is>
+      </c>
+      <c r="X43" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/Sealed%20Genesis%20Terminal</t>
+        </is>
+      </c>
+      <c r="Y43" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=Sealed+Genesis+Terminal</t>
+        </is>
+      </c>
+      <c r="Z43" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/Sealed-Genesis-Terminal</t>
+        </is>
+      </c>
+      <c r="AA43" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=Sealed+Genesis+Terminal&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="43" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="43" t="inlineStr">
+        <is>
+          <t>Glock-18 | Umbral Rabbit (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>8639.776674432</v>
+      </c>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/glock-18-umbral-rabbit/field-tested</t>
+        </is>
+      </c>
+      <c r="F44" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/glock-18-umbral-rabbit?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G44" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/glock-18-umbral-rabbit-field-tested</t>
+        </is>
+      </c>
+      <c r="H44" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I44" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/Glock-18%20%7C%20Umbral%20Rabbit%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J44" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/glock-18-umbral-rabbit-field-tested</t>
+        </is>
+      </c>
+      <c r="K44" s="44" t="n"/>
+      <c r="L44" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M44" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N44" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/glock-18-umbral-rabbit?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O44" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/glock-18-umbral-rabbit/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P44" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/glock-18-umbral-rabbit-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q44" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/Glock-18%20%7C%20Umbral%20Rabbit%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R44" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S44" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/glock-18-umbral-rabbit-field-tested/</t>
+        </is>
+      </c>
+      <c r="T44" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U44" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V44" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/glock-18-umbral-rabbit?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W44" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/glock-18-umbral-rabbit/field-tested</t>
+        </is>
+      </c>
+      <c r="X44" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/Glock-18%20%7C%20Umbral%20Rabbit%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y44" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z44" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/Glock-18-|-Umbral-Rabbit-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA44" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=Glock-18+%7C+Umbral+Rabbit+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="43" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="43" t="inlineStr">
+        <is>
+          <t>M4A1-S | Nitro (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>5071.23951744</v>
+      </c>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/m4a1-s-nitro/field-tested</t>
+        </is>
+      </c>
+      <c r="F45" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/m4a1-s-nitro?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G45" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/m4a1-s-nitro-field-tested</t>
+        </is>
+      </c>
+      <c r="H45" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=M4A1-S+%7C+Nitro+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I45" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/M4A1-S%20%7C%20Nitro%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J45" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/m4a1-s-nitro-field-tested</t>
+        </is>
+      </c>
+      <c r="K45" s="44" t="n"/>
+      <c r="L45" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=M4A1-S+%7C+Nitro+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M45" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=M4A1-S+%7C+Nitro+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N45" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/m4a1-s-nitro?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O45" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/m4a1-s-nitro/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P45" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/m4a1-s-nitro-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q45" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/M4A1-S%20%7C%20Nitro%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R45" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=M4A1-S+%7C+Nitro+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S45" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/m4a1-s-nitro-field-tested/</t>
+        </is>
+      </c>
+      <c r="T45" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=M4A1-S+%7C+Nitro+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U45" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=M4A1-S+%7C+Nitro+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V45" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/m4a1-s-nitro?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W45" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/m4a1-s-nitro/field-tested</t>
+        </is>
+      </c>
+      <c r="X45" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/M4A1-S%20%7C%20Nitro%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y45" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=M4A1-S+%7C+Nitro+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z45" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/M4A1-S-|-Nitro-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA45" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=M4A1-S+%7C+Nitro+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="43" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="43" t="inlineStr">
+        <is>
+          <t>MAC-10 | Sakkaku (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="n">
+        <v>6521.473468128001</v>
+      </c>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/mac-10-sakkaku/field-tested</t>
+        </is>
+      </c>
+      <c r="F46" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/mac-10-sakkaku?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G46" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/mac-10-sakkaku-field-tested</t>
+        </is>
+      </c>
+      <c r="H46" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=MAC-10+%7C+Sakkaku+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I46" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/MAC-10%20%7C%20Sakkaku%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J46" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/mac-10-sakkaku-field-tested</t>
+        </is>
+      </c>
+      <c r="K46" s="44" t="n"/>
+      <c r="L46" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=MAC-10+%7C+Sakkaku+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M46" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=MAC-10+%7C+Sakkaku+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N46" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/mac-10-sakkaku?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O46" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/mac-10-sakkaku/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P46" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/mac-10-sakkaku-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q46" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/MAC-10%20%7C%20Sakkaku%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R46" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=MAC-10+%7C+Sakkaku+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S46" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/mac-10-sakkaku-field-tested/</t>
+        </is>
+      </c>
+      <c r="T46" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=MAC-10+%7C+Sakkaku+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U46" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=MAC-10+%7C+Sakkaku+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V46" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/mac-10-sakkaku?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W46" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/mac-10-sakkaku/field-tested</t>
+        </is>
+      </c>
+      <c r="X46" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/MAC-10%20%7C%20Sakkaku%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y46" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=MAC-10+%7C+Sakkaku+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z46" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/MAC-10-|-Sakkaku-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA46" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=MAC-10+%7C+Sakkaku+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="43" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="43" t="inlineStr">
+        <is>
+          <t>P250 | Re.built (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="n">
+        <v>469.617016384</v>
+      </c>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/p250-rebuilt/field-tested</t>
+        </is>
+      </c>
+      <c r="F47" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/p250-rebuilt?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G47" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/p250-rebuilt-field-tested</t>
+        </is>
+      </c>
+      <c r="H47" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=P250+%7C+Re.built+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I47" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/P250%20%7C%20Re.built%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J47" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/p250-rebuilt-field-tested</t>
+        </is>
+      </c>
+      <c r="K47" s="44" t="n"/>
+      <c r="L47" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=P250+%7C+Re.built+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M47" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=P250+%7C+Re.built+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N47" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/p250-rebuilt?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O47" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/p250-rebuilt/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P47" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/p250-rebuilt-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q47" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/P250%20%7C%20Re.built%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R47" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=P250+%7C+Re.built+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S47" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/p250-rebuilt-field-tested/</t>
+        </is>
+      </c>
+      <c r="T47" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=P250+%7C+Re.built+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U47" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=P250+%7C+Re.built+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V47" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/p250-rebuilt?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W47" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/p250-rebuilt/field-tested</t>
+        </is>
+      </c>
+      <c r="X47" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/P250%20%7C%20Re.built%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y47" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=P250+%7C+Re.built+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z47" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/P250-|-Re.built-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA47" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=P250+%7C+Re.built+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="43" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="43" t="inlineStr">
+        <is>
+          <t>MAG-7 | Foresight (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n">
+        <v>506.74601536</v>
+      </c>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/mag-7-foresight/field-tested</t>
+        </is>
+      </c>
+      <c r="F48" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/mag-7-foresight?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G48" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/mag-7-foresight-field-tested</t>
+        </is>
+      </c>
+      <c r="H48" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=MAG-7+%7C+Foresight+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I48" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/MAG-7%20%7C%20Foresight%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J48" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/mag-7-foresight-field-tested</t>
+        </is>
+      </c>
+      <c r="K48" s="44" t="n"/>
+      <c r="L48" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=MAG-7+%7C+Foresight+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M48" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=MAG-7+%7C+Foresight+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N48" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/mag-7-foresight?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O48" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/mag-7-foresight/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P48" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/mag-7-foresight-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q48" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/MAG-7%20%7C%20Foresight%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R48" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=MAG-7+%7C+Foresight+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S48" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/mag-7-foresight-field-tested/</t>
+        </is>
+      </c>
+      <c r="T48" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=MAG-7+%7C+Foresight+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U48" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=MAG-7+%7C+Foresight+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V48" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/mag-7-foresight?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W48" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/mag-7-foresight/field-tested</t>
+        </is>
+      </c>
+      <c r="X48" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/MAG-7%20%7C%20Foresight%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y48" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=MAG-7+%7C+Foresight+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z48" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/MAG-7-|-Foresight-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA48" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=MAG-7+%7C+Foresight+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="43" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="43" t="inlineStr">
+        <is>
+          <t>Antwerp 2022 Legends Sticker Capsule</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>2087.883899904</v>
+      </c>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/antwerp-2022-legends-sticker-capsule/normal</t>
+        </is>
+      </c>
+      <c r="F49" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/container/antwerp-2022-legends-sticker-capsule</t>
+        </is>
+      </c>
+      <c r="G49" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/antwerp-2022-legends-sticker-capsule</t>
+        </is>
+      </c>
+      <c r="H49" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=Antwerp+2022+Legends+Sticker+Capsule</t>
+        </is>
+      </c>
+      <c r="I49" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/Antwerp%202022%20Legends%20Sticker%20Capsule</t>
+        </is>
+      </c>
+      <c r="J49" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/antwerp-2022-legends-sticker-capsule</t>
+        </is>
+      </c>
+      <c r="K49" s="44" t="n"/>
+      <c r="L49" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=Antwerp+2022+Legends+Sticker+Capsule&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=normal</t>
+        </is>
+      </c>
+      <c r="M49" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=Antwerp+2022+Legends+Sticker+Capsule</t>
+        </is>
+      </c>
+      <c r="N49" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/antwerp-2022-legends-sticker-capsule?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=normal</t>
+        </is>
+      </c>
+      <c r="O49" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/antwerp-2022-legends-sticker-capsule</t>
+        </is>
+      </c>
+      <c r="P49" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/antwerp-2022-legends-sticker-capsule/</t>
+        </is>
+      </c>
+      <c r="Q49" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/Antwerp%202022%20Legends%20Sticker%20Capsule</t>
+        </is>
+      </c>
+      <c r="R49" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=Antwerp+2022+Legends+Sticker+Capsule&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S49" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/antwerp-2022-legends-sticker-capsule/</t>
+        </is>
+      </c>
+      <c r="T49" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=Antwerp+2022+Legends+Sticker+Capsule</t>
+        </is>
+      </c>
+      <c r="U49" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=Antwerp+2022+Legends+Sticker+Capsule</t>
+        </is>
+      </c>
+      <c r="V49" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/antwerp-2022-legends-sticker-capsule</t>
+        </is>
+      </c>
+      <c r="W49" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/antwerp-2022-legends-sticker-capsule</t>
+        </is>
+      </c>
+      <c r="X49" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/Antwerp%202022%20Legends%20Sticker%20Capsule</t>
+        </is>
+      </c>
+      <c r="Y49" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=Antwerp+2022+Legends+Sticker+Capsule</t>
+        </is>
+      </c>
+      <c r="Z49" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/Antwerp-2022-Legends-Sticker-Capsule</t>
+        </is>
+      </c>
+      <c r="AA49" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=Antwerp+2022+Legends+Sticker+Capsule&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="43" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="43" t="inlineStr">
+        <is>
+          <t>G3SG1 | Red Jasper (Factory New)</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n">
+        <v>392.151410496</v>
+      </c>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/g3sg1-red-jasper/factory-new</t>
+        </is>
+      </c>
+      <c r="F50" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/g3sg1-red-jasper?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G50" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/g3sg1-red-jasper-factory-new</t>
+        </is>
+      </c>
+      <c r="H50" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=G3SG1+%7C+Red+Jasper+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I50" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/G3SG1%20%7C%20Red%20Jasper%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J50" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/g3sg1-red-jasper-factory-new</t>
+        </is>
+      </c>
+      <c r="K50" s="44" t="n"/>
+      <c r="L50" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=G3SG1+%7C+Red+Jasper+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M50" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=G3SG1+%7C+Red+Jasper+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N50" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/g3sg1-red-jasper?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O50" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/g3sg1-red-jasper/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P50" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/g3sg1-red-jasper-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q50" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/G3SG1%20%7C%20Red%20Jasper%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R50" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=G3SG1+%7C+Red+Jasper+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S50" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/g3sg1-red-jasper-factory-new/</t>
+        </is>
+      </c>
+      <c r="T50" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=G3SG1+%7C+Red+Jasper+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U50" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=G3SG1+%7C+Red+Jasper+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V50" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/g3sg1-red-jasper?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W50" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/g3sg1-red-jasper/factory-new</t>
+        </is>
+      </c>
+      <c r="X50" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/G3SG1%20%7C%20Red%20Jasper%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y50" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=G3SG1+%7C+Red+Jasper+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z50" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/G3SG1-|-Red-Jasper-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA50" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=G3SG1+%7C+Red+Jasper+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="43" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="43" t="inlineStr">
+        <is>
+          <t>MAC-10 | Ensnared (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="n">
+        <v>441.571342208</v>
+      </c>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/mac-10-ensnared/field-tested</t>
+        </is>
+      </c>
+      <c r="F51" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/mac-10-ensnared?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G51" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/mac-10-ensnared-field-tested</t>
+        </is>
+      </c>
+      <c r="H51" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=MAC-10+%7C+Ensnared+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I51" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/MAC-10%20%7C%20Ensnared%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J51" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/mac-10-ensnared-field-tested</t>
+        </is>
+      </c>
+      <c r="K51" s="44" t="n"/>
+      <c r="L51" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=MAC-10+%7C+Ensnared+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M51" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=MAC-10+%7C+Ensnared+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N51" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/mac-10-ensnared?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O51" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/mac-10-ensnared/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P51" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/mac-10-ensnared-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q51" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/MAC-10%20%7C%20Ensnared%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R51" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=MAC-10+%7C+Ensnared+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S51" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/mac-10-ensnared-field-tested/</t>
+        </is>
+      </c>
+      <c r="T51" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=MAC-10+%7C+Ensnared+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U51" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=MAC-10+%7C+Ensnared+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V51" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/mac-10-ensnared?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W51" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/mac-10-ensnared/field-tested</t>
+        </is>
+      </c>
+      <c r="X51" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/MAC-10%20%7C%20Ensnared%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y51" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=MAC-10+%7C+Ensnared+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z51" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/MAC-10-|-Ensnared-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA51" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=MAC-10+%7C+Ensnared+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="43" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="43" t="inlineStr">
+        <is>
+          <t>★ Skeleton Knife | Doppler (Factory New)</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>173399.84045184</v>
+      </c>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/skeleton-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="F52" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/skeleton-knife-doppler?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G52" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/skeleton-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="H52" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I52" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/%E2%98%85%20Skeleton%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J52" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/skeleton-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="K52" s="44" t="n"/>
+      <c r="L52" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M52" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N52" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/skeleton-knife-doppler?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O52" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/skeleton-knife-doppler/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P52" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/skeleton-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q52" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/%E2%98%85%20Skeleton%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R52" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S52" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/skeleton-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="T52" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U52" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V52" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/skeleton-knife-doppler?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W52" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/skeleton-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="X52" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/%E2%98%85%20Skeleton%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y52" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z52" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/★-Skeleton-Knife-|-Doppler-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA52" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=%E2%98%85+Skeleton+Knife+%7C+Doppler+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="43" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="43" t="inlineStr">
+        <is>
+          <t>AK-47 | Case Hardened (Factory New)</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="n">
+        <v>142069.413448704</v>
+      </c>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/ak-47-case-hardened/factory-new</t>
+        </is>
+      </c>
+      <c r="F53" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/ak-47-case-hardened?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G53" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/ak-47-case-hardened-factory-new</t>
+        </is>
+      </c>
+      <c r="H53" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=AK-47+%7C+Case+Hardened+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I53" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/AK-47%20%7C%20Case%20Hardened%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J53" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/ak-47-case-hardened-factory-new</t>
+        </is>
+      </c>
+      <c r="K53" s="44" t="n"/>
+      <c r="L53" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=AK-47+%7C+Case+Hardened+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M53" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=AK-47+%7C+Case+Hardened+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N53" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/ak-47-case-hardened?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O53" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/ak-47-case-hardened/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P53" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/ak-47-case-hardened-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q53" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/AK-47%20%7C%20Case%20Hardened%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R53" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=AK-47+%7C+Case+Hardened+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S53" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/ak-47-case-hardened-factory-new/</t>
+        </is>
+      </c>
+      <c r="T53" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=AK-47+%7C+Case+Hardened+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U53" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=AK-47+%7C+Case+Hardened+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V53" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/ak-47-case-hardened?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W53" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/ak-47-case-hardened/factory-new</t>
+        </is>
+      </c>
+      <c r="X53" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/AK-47%20%7C%20Case%20Hardened%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y53" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=AK-47+%7C+Case+Hardened+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z53" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/AK-47-|-Case-Hardened-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA53" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=AK-47+%7C+Case+Hardened+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="43" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="43" t="inlineStr">
+        <is>
+          <t>★ Stiletto Knife | Doppler (Factory New)</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="n">
+        <v>137535.123676416</v>
+      </c>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/stiletto-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="F54" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/stiletto-knife-doppler?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G54" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/stiletto-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="H54" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I54" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/%E2%98%85%20Stiletto%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J54" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/stiletto-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="K54" s="44" t="n"/>
+      <c r="L54" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M54" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N54" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/stiletto-knife-doppler?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O54" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/stiletto-knife-doppler/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P54" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/stiletto-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q54" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/%E2%98%85%20Stiletto%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R54" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S54" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/stiletto-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="T54" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U54" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V54" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/stiletto-knife-doppler?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W54" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/stiletto-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="X54" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/%E2%98%85%20Stiletto%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y54" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z54" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/★-Stiletto-Knife-|-Doppler-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA54" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=%E2%98%85+Stiletto+Knife+%7C+Doppler+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="43" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="43" t="inlineStr">
+        <is>
+          <t>★ Talon Knife | Doppler (Factory New)</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>135609.06454368</v>
+      </c>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/talon-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="F55" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/talon-knife-doppler?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G55" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/talon-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="H55" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I55" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/%E2%98%85%20Talon%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J55" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/talon-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="K55" s="44" t="n"/>
+      <c r="L55" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M55" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N55" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/talon-knife-doppler?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O55" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/talon-knife-doppler/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P55" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/talon-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q55" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/%E2%98%85%20Talon%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R55" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S55" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/talon-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="T55" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U55" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V55" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/talon-knife-doppler?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W55" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/talon-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="X55" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/%E2%98%85%20Talon%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y55" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z55" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/★-Talon-Knife-|-Doppler-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA55" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=%E2%98%85+Talon+Knife+%7C+Doppler+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="43" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="43" t="inlineStr">
+        <is>
+          <t>★ Karambit | Gamma Doppler (Factory New)</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="n">
+        <v>131620.675888128</v>
+      </c>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/karambit-gamma-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="F56" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/karambit-gamma-doppler?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G56" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/karambit-gamma-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="H56" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I56" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/%E2%98%85%20Karambit%20%7C%20Gamma%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J56" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/karambit-gamma-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="K56" s="44" t="n"/>
+      <c r="L56" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M56" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N56" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/karambit-gamma-doppler?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O56" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/karambit-gamma-doppler/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P56" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/karambit-gamma-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q56" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/%E2%98%85%20Karambit%20%7C%20Gamma%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R56" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S56" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/karambit-gamma-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="T56" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U56" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V56" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/karambit-gamma-doppler?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W56" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/karambit-gamma-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="X56" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/%E2%98%85%20Karambit%20%7C%20Gamma%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y56" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z56" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/★-Karambit-|-Gamma-Doppler-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA56" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=%E2%98%85+Karambit+%7C+Gamma+Doppler+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="43" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="43" t="inlineStr">
+        <is>
+          <t>★ Karambit | Fade (Factory New)</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="n">
+        <v>125739.2302848</v>
+      </c>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/karambit-fade/factory-new</t>
+        </is>
+      </c>
+      <c r="F57" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/karambit-fade?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G57" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/karambit-fade-factory-new</t>
+        </is>
+      </c>
+      <c r="H57" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I57" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/%E2%98%85%20Karambit%20%7C%20Fade%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J57" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/karambit-fade-factory-new</t>
+        </is>
+      </c>
+      <c r="K57" s="44" t="n"/>
+      <c r="L57" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M57" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N57" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/karambit-fade?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O57" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/karambit-fade/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P57" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/karambit-fade-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q57" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/%E2%98%85%20Karambit%20%7C%20Fade%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R57" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S57" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/karambit-fade-factory-new/</t>
+        </is>
+      </c>
+      <c r="T57" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U57" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V57" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/karambit-fade?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W57" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/karambit-fade/factory-new</t>
+        </is>
+      </c>
+      <c r="X57" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/%E2%98%85%20Karambit%20%7C%20Fade%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y57" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z57" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/★-Karambit-|-Fade-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA57" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=%E2%98%85+Karambit+%7C+Fade+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="43" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="43" t="inlineStr">
+        <is>
+          <t>AWP | Dragon Lore (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="n">
+        <v>123839.775794688</v>
+      </c>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/awp-dragon-lore/field-tested</t>
+        </is>
+      </c>
+      <c r="F58" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/awp-dragon-lore?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G58" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/awp-dragon-lore-field-tested</t>
+        </is>
+      </c>
+      <c r="H58" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=AWP+%7C+Dragon+Lore+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I58" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/AWP%20%7C%20Dragon%20Lore%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J58" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/awp-dragon-lore-field-tested</t>
+        </is>
+      </c>
+      <c r="K58" s="44" t="n"/>
+      <c r="L58" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=AWP+%7C+Dragon+Lore+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M58" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=AWP+%7C+Dragon+Lore+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N58" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/awp-dragon-lore?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O58" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/awp-dragon-lore/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P58" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/awp-dragon-lore-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q58" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/AWP%20%7C%20Dragon%20Lore%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R58" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=AWP+%7C+Dragon+Lore+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S58" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/awp-dragon-lore-field-tested/</t>
+        </is>
+      </c>
+      <c r="T58" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=AWP+%7C+Dragon+Lore+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U58" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=AWP+%7C+Dragon+Lore+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V58" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/awp-dragon-lore?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W58" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/awp-dragon-lore/field-tested</t>
+        </is>
+      </c>
+      <c r="X58" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/AWP%20%7C%20Dragon%20Lore%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y58" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=AWP+%7C+Dragon+Lore+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z58" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/AWP-|-Dragon-Lore-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA58" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=AWP+%7C+Dragon+Lore+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="43" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="43" t="inlineStr">
+        <is>
+          <t>★ Sport Gloves | Arid (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>115814.372332032</v>
+      </c>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/sport-gloves-arid/field-tested</t>
+        </is>
+      </c>
+      <c r="F59" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/glove/sport-gloves-arid?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G59" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/sport-gloves-arid-field-tested</t>
+        </is>
+      </c>
+      <c r="H59" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I59" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/%E2%98%85%20Sport%20Gloves%20%7C%20Arid%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J59" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/sport-gloves-arid-field-tested</t>
+        </is>
+      </c>
+      <c r="K59" s="44" t="n"/>
+      <c r="L59" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M59" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N59" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/sport-gloves-arid?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O59" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/sport-gloves-arid/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P59" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/sport-gloves-arid-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q59" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/%E2%98%85%20Sport%20Gloves%20%7C%20Arid%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R59" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S59" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/sport-gloves-arid-field-tested/</t>
+        </is>
+      </c>
+      <c r="T59" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U59" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V59" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/sport-gloves-arid?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W59" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/sport-gloves-arid/field-tested</t>
+        </is>
+      </c>
+      <c r="X59" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/%E2%98%85%20Sport%20Gloves%20%7C%20Arid%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y59" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z59" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/★-Sport-Gloves-|-Arid-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA59" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=%E2%98%85+Sport+Gloves+%7C+Arid+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="43" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="43" t="inlineStr">
+        <is>
+          <t>★ Flip Knife | Doppler (Factory New)</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="n">
+        <v>106570.391327616</v>
+      </c>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/flip-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="F60" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/flip-knife-doppler?variant=factory-new</t>
+        </is>
+      </c>
+      <c r="G60" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/flip-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="H60" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="I60" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/%E2%98%85%20Flip%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="J60" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/flip-knife-doppler-factory-new</t>
+        </is>
+      </c>
+      <c r="K60" s="44" t="n"/>
+      <c r="L60" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Factory+New</t>
+        </is>
+      </c>
+      <c r="M60" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="N60" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/flip-knife-doppler?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=factory-new</t>
+        </is>
+      </c>
+      <c r="O60" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/flip-knife-doppler/normal-factory-new</t>
+        </is>
+      </c>
+      <c r="P60" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/flip-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="Q60" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/%E2%98%85%20Flip%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="R60" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S60" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/flip-knife-doppler-factory-new/</t>
+        </is>
+      </c>
+      <c r="T60" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="U60" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="V60" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/flip-knife-doppler?exterior=fa</t>
+        </is>
+      </c>
+      <c r="W60" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/flip-knife-doppler/factory-new</t>
+        </is>
+      </c>
+      <c r="X60" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/%E2%98%85%20Flip%20Knife%20%7C%20Doppler%20%28Factory%20New%29</t>
+        </is>
+      </c>
+      <c r="Y60" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29</t>
+        </is>
+      </c>
+      <c r="Z60" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/★-Flip-Knife-|-Doppler-(Factory New)</t>
+        </is>
+      </c>
+      <c r="AA60" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=%E2%98%85+Flip+Knife+%7C+Doppler+%28Factory+New%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="43" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="43" t="inlineStr">
+        <is>
+          <t>MP9 | Starlight Protector (Field-Tested)</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="n">
+        <v>102409.734859488</v>
+      </c>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="43" t="inlineStr">
+        <is>
+          <t>https://csgoskins.gg/items/mp9-starlight-protector/field-tested</t>
+        </is>
+      </c>
+      <c r="F61" s="25" t="inlineStr">
+        <is>
+          <t>https://pricempire.com/cs2-items/skin/mp9-starlight-protector?variant=field-tested</t>
+        </is>
+      </c>
+      <c r="G61" s="43" t="inlineStr">
+        <is>
+          <t>https://www.steamanalyst.com/skin/mp9-starlight-protector-field-tested</t>
+        </is>
+      </c>
+      <c r="H61" s="44" t="inlineStr">
+        <is>
+          <t>https://www.haloskins.com/market?keyword=MP9+%7C+Starlight+Protector+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="I61" s="44" t="inlineStr">
+        <is>
+          <t>https://aim.market/en/buy/csgo/MP9%20%7C%20Starlight%20Protector%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="J61" s="44" t="inlineStr">
+        <is>
+          <t>https://avan.market/market/cs/mp9-starlight-protector-field-tested</t>
+        </is>
+      </c>
+      <c r="K61" s="44" t="n"/>
+      <c r="L61" s="44" t="inlineStr">
+        <is>
+          <t>https://cs.money/market/buy/?search=MP9+%7C+Starlight+Protector+%28Field-Tested%29&amp;sort=price&amp;order=asc&amp;isStatTrak=false&amp;isSouvenir=false&amp;exterior=Field-Tested</t>
+        </is>
+      </c>
+      <c r="M61" s="44" t="inlineStr">
+        <is>
+          <t>https://csfloat.com/search?sort_by=lowest_price&amp;type=buy_now&amp;market_hash_name=MP9+%7C+Starlight+Protector+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="N61" s="44" t="inlineStr">
+        <is>
+          <t>https://dmarket.com/csgo-skins/product-card/mp9-starlight-protector?sort-type=5&amp;category_0=not_stattrak_tm&amp;category_1=not_souvenir&amp;exterior=field-tested</t>
+        </is>
+      </c>
+      <c r="O61" s="44" t="inlineStr">
+        <is>
+          <t>https://exeskins.com/item/mp9-starlight-protector/normal-field-tested</t>
+        </is>
+      </c>
+      <c r="P61" s="44" t="inlineStr">
+        <is>
+          <t>https://lis-skins.com/market/csgo/mp9-starlight-protector-field-tested/</t>
+        </is>
+      </c>
+      <c r="Q61" s="44" t="inlineStr">
+        <is>
+          <t>https://market.csgo.com/en/MP9%20%7C%20Starlight%20Protector%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="R61" s="44" t="inlineStr">
+        <is>
+          <t>https://shadowpay.com/csgo-items?search=MP9+%7C+Starlight+Protector+%28Field-Tested%29&amp;is_stattrak=0&amp;sort_column=price&amp;sort_dir=asc</t>
+        </is>
+      </c>
+      <c r="S61" s="44" t="inlineStr">
+        <is>
+          <t>https://app.skin.land/market/csgo/mp9-starlight-protector-field-tested/</t>
+        </is>
+      </c>
+      <c r="T61" s="44" t="inlineStr">
+        <is>
+          <t>https://skinbaron.de/csgo?search=MP9+%7C+Starlight+Protector+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="U61" s="44" t="inlineStr">
+        <is>
+          <t>https://skin.place/buy-cs2-skins?search=MP9+%7C+Starlight+Protector+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="V61" s="44" t="inlineStr">
+        <is>
+          <t>https://skins.com/item/mp9-starlight-protector?exterior=fi</t>
+        </is>
+      </c>
+      <c r="W61" s="44" t="inlineStr">
+        <is>
+          <t>https://skinswap.com/skins/mp9-starlight-protector/field-tested</t>
+        </is>
+      </c>
+      <c r="X61" s="44" t="inlineStr">
+        <is>
+          <t>https://skinvault.gg/buy-csgo-skins/MP9%20%7C%20Starlight%20Protector%20%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Y61" s="44" t="inlineStr">
+        <is>
+          <t>https://tradeit.gg/csgo/store?search=MP9+%7C+Starlight+Protector+%28Field-Tested%29</t>
+        </is>
+      </c>
+      <c r="Z61" s="44" t="inlineStr">
+        <is>
+          <t>https://www.uuskins.com/items/MP9-|-Starlight-Protector-(Field-Tested)</t>
+        </is>
+      </c>
+      <c r="AA61" s="44" t="inlineStr">
+        <is>
+          <t>https://waxpeer.com/?sort=ASC&amp;order=price&amp;all=0&amp;skip=0&amp;game=csgo&amp;search=MP9+%7C+Starlight+Protector+%28Field-Tested%29&amp;exact=1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>